<commit_message>
Page 7: 34 rows incl PS5-78-01, restored original styling + macro + filter
</commit_message>
<xml_diff>
--- a/EXCEL/7 - COMPLETE.xlsx
+++ b/EXCEL/7 - COMPLETE.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIDMAP" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'7 · COMPLETE'!$A$2:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'7 · COMPLETE'!$A$2:$G$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1113,7 +1113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2044,34 +2044,65 @@
       <c r="G34" s="64" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="78" t="n">
-        <v>33</v>
+      <c r="A35" s="82" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
       </c>
       <c r="B35" s="80" t="inlineStr">
         <is>
+          <t>PS5-78-01 - Lifting and handling equipment</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>PS5 - Milestone E</t>
+        </is>
+      </c>
+      <c r="E35" s="65" t="inlineStr">
+        <is>
+          <t>PARTIAL(05-03-2026)</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="64" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="78" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B36" s="80" t="inlineStr">
+        <is>
           <t>PS5-91-01 - Multicore cables &amp; JB</t>
         </is>
       </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="D35" s="24" t="inlineStr">
+      <c r="D36" s="24" t="inlineStr">
         <is>
           <t>PS5 - Milestone A</t>
         </is>
       </c>
-      <c r="E35" s="67" t="inlineStr">
+      <c r="E36" s="67" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="F35" s="23" t="inlineStr"/>
-      <c r="G35" s="64" t="inlineStr"/>
+      <c r="F36" s="23" t="inlineStr"/>
+      <c r="G36" s="64" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G35"/>
+  <autoFilter ref="A2:G36"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>